<commit_message>
Revise language from "No S/THO Oversight" to "Separate Oversight"; update broken/missing links; update MT data
</commit_message>
<xml_diff>
--- a/updatedMemberData.xlsx
+++ b/updatedMemberData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madmarshall/Documents/medicaidOversightMap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82BD0D06-82C2-EF45-8B5A-FBC27D05E168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB0BD0E-7263-EC42-BB7D-4AA520EB14B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7220" yWindow="660" windowWidth="21400" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7100" yWindow="660" windowWidth="21400" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1958" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1960" uniqueCount="494">
   <si>
     <t>Oversight?</t>
   </si>
@@ -1499,6 +1499,27 @@
   </si>
   <si>
     <t>Louisiana</t>
+  </si>
+  <si>
+    <t>https://www.dpbh.nv.gov/about/organizational-charts/</t>
+  </si>
+  <si>
+    <t>https://health.mo.gov/about/pdf/org-chart-ada.pdf</t>
+  </si>
+  <si>
+    <t>https://www.nmhealth.org/about/</t>
+  </si>
+  <si>
+    <t>https://dph.sc.gov/sites/scdph/files/Library/00029-ENG-CR.pdf</t>
+  </si>
+  <si>
+    <t>https://dph.georgia.gov/about-dph</t>
+  </si>
+  <si>
+    <t>https://www.chfs.ky.gov/agencies/Pages/default.aspx</t>
+  </si>
+  <si>
+    <t>https://www.tn.gov/health/dept.html</t>
   </si>
 </sst>
 </file>
@@ -1674,7 +1695,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1696,23 +1717,15 @@
     <xf numFmtId="22" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="22" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="22" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="22" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1853,21 +1866,21 @@
     <sortCondition descending="1" ref="A1:A58"/>
   </sortState>
   <tableColumns count="21">
-    <tableColumn id="24" xr3:uid="{EC3A8AE4-1AEA-44FE-9DAE-C845A25235D5}" name="Oversight?" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{80BFFD16-634B-644C-BC67-0E0C16458147}" name="jurisdictionName" dataDxfId="5"/>
+    <tableColumn id="24" xr3:uid="{EC3A8AE4-1AEA-44FE-9DAE-C845A25235D5}" name="Oversight?" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{80BFFD16-634B-644C-BC67-0E0C16458147}" name="jurisdictionName" dataDxfId="12"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Account Name"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Agency Structure"/>
-    <tableColumn id="23" xr3:uid="{091B2DD4-B1BA-4A29-9F94-96F9DC3BAAB3}" name="Public Health Website" dataDxfId="4" dataCellStyle="Hyperlink"/>
-    <tableColumn id="25" xr3:uid="{AF3B510E-B66B-4682-A68A-7103145FD741}" name="HHS or Medicaid Context " dataDxfId="3" dataCellStyle="Hyperlink"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Governor Term Year" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Acronym" dataDxfId="1"/>
+    <tableColumn id="23" xr3:uid="{091B2DD4-B1BA-4A29-9F94-96F9DC3BAAB3}" name="Public Health Website" dataDxfId="11" dataCellStyle="Hyperlink"/>
+    <tableColumn id="25" xr3:uid="{AF3B510E-B66B-4682-A68A-7103145FD741}" name="HHS or Medicaid Context " dataDxfId="10" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Governor Term Year" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Acronym" dataDxfId="8"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Governance Classification"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="S/THO"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="S/THO Designee"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="S/THO Acting"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="S/THO Assistant"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="City"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Org Chart" dataDxfId="0"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Org Chart" dataDxfId="7"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Secretary of Health"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Population"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="PHAB Accreditation"/>
@@ -1886,21 +1899,21 @@
     <sortCondition ref="C1:C58"/>
   </sortState>
   <tableColumns count="21">
-    <tableColumn id="24" xr3:uid="{14C78B0C-CC4B-CF46-9A7C-80025A9DF37D}" name="Oversight?" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{6CBE6995-E45E-3049-8744-E0D6CCBBA85B}" name="jurisdictionName" dataDxfId="12"/>
+    <tableColumn id="24" xr3:uid="{14C78B0C-CC4B-CF46-9A7C-80025A9DF37D}" name="Oversight?" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{6CBE6995-E45E-3049-8744-E0D6CCBBA85B}" name="jurisdictionName" dataDxfId="5"/>
     <tableColumn id="5" xr3:uid="{ABF7AE7E-A482-594D-A5CB-B4905C32B62F}" name="Account Name"/>
     <tableColumn id="8" xr3:uid="{BF737C6C-A012-604E-A01C-BCFB91745840}" name="Agency Structure"/>
-    <tableColumn id="23" xr3:uid="{608D6F1D-623F-1C46-A561-376D2FF08802}" name="Public Health Website" dataDxfId="11" dataCellStyle="Hyperlink"/>
-    <tableColumn id="25" xr3:uid="{7589D836-3A5F-7245-BA28-2ECAE78D012C}" name="HHS or Medicaid Context " dataDxfId="10" dataCellStyle="Hyperlink"/>
-    <tableColumn id="6" xr3:uid="{95DCC688-5259-4A49-930B-C3CC0DEC12A1}" name="Governor Term Year" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{0204E4C1-D1DD-544F-8D61-3FF5C9921AA5}" name="Acronym" dataDxfId="8"/>
+    <tableColumn id="23" xr3:uid="{608D6F1D-623F-1C46-A561-376D2FF08802}" name="Public Health Website" dataDxfId="4" dataCellStyle="Hyperlink"/>
+    <tableColumn id="25" xr3:uid="{7589D836-3A5F-7245-BA28-2ECAE78D012C}" name="HHS or Medicaid Context " dataDxfId="3" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{95DCC688-5259-4A49-930B-C3CC0DEC12A1}" name="Governor Term Year" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{0204E4C1-D1DD-544F-8D61-3FF5C9921AA5}" name="Acronym" dataDxfId="1"/>
     <tableColumn id="9" xr3:uid="{ACCB8137-D23C-A946-8E75-567466A7F46C}" name="Governance Classification"/>
     <tableColumn id="10" xr3:uid="{7DCBF5BA-5DF1-0047-AE0D-A6E10097AAEC}" name="S/THO"/>
     <tableColumn id="11" xr3:uid="{1A2764D9-A525-1B44-B6ED-2AA6B8858981}" name="S/THO Designee"/>
     <tableColumn id="12" xr3:uid="{A681CC24-8158-CD49-8463-FE64CB9B7E72}" name="S/THO Acting"/>
     <tableColumn id="13" xr3:uid="{AD1D389E-A518-B442-8CA6-24244C29E7BB}" name="S/THO Assistant"/>
     <tableColumn id="14" xr3:uid="{4329E990-607A-A842-94A4-0B9A7726AEFA}" name="City"/>
-    <tableColumn id="15" xr3:uid="{95704B20-B1E8-5E4D-BE79-A10A24760E8F}" name="Org Chart" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{95704B20-B1E8-5E4D-BE79-A10A24760E8F}" name="Org Chart" dataDxfId="0"/>
     <tableColumn id="16" xr3:uid="{C1E947F7-D643-6B4D-8B70-FCF6D199B1B7}" name="Secretary of Health"/>
     <tableColumn id="17" xr3:uid="{AB12B992-E9C8-5143-B983-304420EB6603}" name="Population"/>
     <tableColumn id="18" xr3:uid="{4DBDC531-DAC6-5E48-8329-7F795ECC5EBD}" name="PHAB Accreditation"/>
@@ -2237,6 +2250,7 @@
     <col min="3" max="4" width="26.5" customWidth="1"/>
     <col min="5" max="5" width="37.83203125" style="5" customWidth="1"/>
     <col min="6" max="6" width="30" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5" customWidth="1"/>
     <col min="8" max="8" width="26.33203125" customWidth="1"/>
     <col min="9" max="9" width="23.5" style="1" customWidth="1"/>
     <col min="10" max="13" width="14" style="1" customWidth="1"/>
@@ -2328,7 +2342,7 @@
         <v>260</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>311</v>
+        <v>492</v>
       </c>
       <c r="F2" s="7"/>
       <c r="G2" s="1" t="s">
@@ -2378,7 +2392,7 @@
       <c r="A3" s="14" t="s">
         <v>309</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="24" t="s">
         <v>453</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -2387,11 +2401,11 @@
       <c r="D3" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="E3" s="36" t="s">
+      <c r="E3" s="29" t="s">
         <v>336</v>
       </c>
       <c r="F3" s="7"/>
-      <c r="G3" s="37" t="s">
+      <c r="G3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="H3" s="1" t="s">
@@ -2438,7 +2452,7 @@
       <c r="A4" s="14" t="s">
         <v>309</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="24" t="s">
         <v>458</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -2447,11 +2461,11 @@
       <c r="D4" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="E4" s="36" t="s">
+      <c r="E4" s="29" t="s">
         <v>349</v>
       </c>
       <c r="F4" s="7"/>
-      <c r="G4" s="37" t="s">
+      <c r="G4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="H4" s="1" t="s">
@@ -2602,7 +2616,7 @@
       <c r="A7" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="24" t="s">
         <v>469</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -2999,10 +3013,10 @@
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A14" s="15" t="s">
-        <v>258</v>
-      </c>
-      <c r="B14" s="29" t="s">
+      <c r="A14" s="14" t="s">
+        <v>309</v>
+      </c>
+      <c r="B14" s="24" t="s">
         <v>457</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -3056,7 +3070,7 @@
       <c r="A15" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="24" t="s">
         <v>459</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -3066,7 +3080,7 @@
         <v>260</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>355</v>
+        <v>487</v>
       </c>
       <c r="F15" s="7"/>
       <c r="G15" s="1" t="s">
@@ -3114,7 +3128,7 @@
       <c r="A16" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="24" t="s">
         <v>460</v>
       </c>
       <c r="C16" s="1" t="s">
@@ -3171,7 +3185,7 @@
       <c r="A17" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="24" t="s">
         <v>464</v>
       </c>
       <c r="C17" s="1" t="s">
@@ -3228,7 +3242,7 @@
       <c r="A18" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="24" t="s">
         <v>466</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -3278,7 +3292,7 @@
       <c r="A19" s="15" t="s">
         <v>403</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="24" t="s">
         <v>474</v>
       </c>
       <c r="C19" s="1" t="s">
@@ -3335,7 +3349,7 @@
       <c r="A20" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="24" t="s">
         <v>483</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -3389,7 +3403,7 @@
       <c r="A21" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="24" t="s">
         <v>484</v>
       </c>
       <c r="C21" s="1" t="s">
@@ -3448,7 +3462,7 @@
       <c r="A22" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="24" t="s">
         <v>485</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -3507,7 +3521,7 @@
       <c r="A23" s="17" t="s">
         <v>390</v>
       </c>
-      <c r="B23" s="29" t="s">
+      <c r="B23" s="24" t="s">
         <v>472</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -3555,7 +3569,7 @@
       <c r="A24" s="17" t="s">
         <v>390</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="24" t="s">
         <v>473</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -4068,7 +4082,9 @@
       <c r="D33" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E33" s="1"/>
+      <c r="E33" s="4" t="s">
+        <v>491</v>
+      </c>
       <c r="F33" s="8"/>
       <c r="G33" s="1" t="s">
         <v>24</v>
@@ -4395,7 +4411,7 @@
       <c r="A39" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B39" s="29" t="s">
+      <c r="B39" s="24" t="s">
         <v>454</v>
       </c>
       <c r="C39" s="1" t="s">
@@ -4452,7 +4468,7 @@
       <c r="A40" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B40" s="29" t="s">
+      <c r="B40" s="24" t="s">
         <v>455</v>
       </c>
       <c r="C40" s="1" t="s">
@@ -4509,7 +4525,7 @@
       <c r="A41" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="24" t="s">
         <v>456</v>
       </c>
       <c r="C41" s="1" t="s">
@@ -4519,7 +4535,7 @@
         <v>22</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>127</v>
+        <v>488</v>
       </c>
       <c r="F41" s="7"/>
       <c r="G41" s="1" t="s">
@@ -4563,7 +4579,7 @@
       <c r="A42" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B42" s="29" t="s">
+      <c r="B42" s="24" t="s">
         <v>461</v>
       </c>
       <c r="C42" s="1" t="s">
@@ -4620,7 +4636,7 @@
       <c r="A43" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B43" s="24" t="s">
         <v>462</v>
       </c>
       <c r="C43" s="1" t="s">
@@ -4630,7 +4646,7 @@
         <v>22</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>140</v>
+        <v>489</v>
       </c>
       <c r="F43" s="7"/>
       <c r="G43" s="1" t="s">
@@ -4680,7 +4696,7 @@
       <c r="A44" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B44" s="29" t="s">
+      <c r="B44" s="24" t="s">
         <v>463</v>
       </c>
       <c r="C44" s="1" t="s">
@@ -4734,7 +4750,7 @@
       <c r="A45" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B45" s="29" t="s">
+      <c r="B45" s="24" t="s">
         <v>465</v>
       </c>
       <c r="C45" s="1" t="s">
@@ -4791,7 +4807,7 @@
       <c r="A46" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B46" s="29" t="s">
+      <c r="B46" s="24" t="s">
         <v>467</v>
       </c>
       <c r="C46" s="1" t="s">
@@ -4848,7 +4864,7 @@
       <c r="A47" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B47" s="24" t="s">
         <v>468</v>
       </c>
       <c r="C47" s="1" t="s">
@@ -4902,7 +4918,7 @@
       <c r="A48" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="29" t="s">
+      <c r="B48" s="24" t="s">
         <v>470</v>
       </c>
       <c r="C48" s="1" t="s">
@@ -4959,7 +4975,7 @@
       <c r="A49" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B49" s="29" t="s">
+      <c r="B49" s="24" t="s">
         <v>471</v>
       </c>
       <c r="C49" s="1" t="s">
@@ -5009,7 +5025,7 @@
       <c r="A50" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="29" t="s">
+      <c r="B50" s="24" t="s">
         <v>475</v>
       </c>
       <c r="C50" s="1" t="s">
@@ -5019,7 +5035,7 @@
         <v>22</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>179</v>
+        <v>490</v>
       </c>
       <c r="F50" s="7"/>
       <c r="G50" s="1" t="s">
@@ -5069,7 +5085,7 @@
       <c r="A51" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B51" s="29" t="s">
+      <c r="B51" s="24" t="s">
         <v>476</v>
       </c>
       <c r="C51" s="1" t="s">
@@ -5126,7 +5142,7 @@
       <c r="A52" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B52" s="29" t="s">
+      <c r="B52" s="24" t="s">
         <v>477</v>
       </c>
       <c r="C52" s="1" t="s">
@@ -5135,7 +5151,9 @@
       <c r="D52" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E52" s="1"/>
+      <c r="E52" s="4" t="s">
+        <v>493</v>
+      </c>
       <c r="F52" s="8"/>
       <c r="G52" s="1" t="s">
         <v>24</v>
@@ -5175,7 +5193,7 @@
       <c r="A53" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B53" s="29" t="s">
+      <c r="B53" s="24" t="s">
         <v>478</v>
       </c>
       <c r="C53" s="1" t="s">
@@ -5230,7 +5248,7 @@
       <c r="A54" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B54" s="29" t="s">
+      <c r="B54" s="24" t="s">
         <v>479</v>
       </c>
       <c r="C54" s="1" t="s">
@@ -5283,7 +5301,7 @@
       <c r="A55" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B55" s="29" t="s">
+      <c r="B55" s="24" t="s">
         <v>480</v>
       </c>
       <c r="C55" s="1" t="s">
@@ -5340,7 +5358,7 @@
       <c r="A56" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B56" s="29" t="s">
+      <c r="B56" s="24" t="s">
         <v>481</v>
       </c>
       <c r="C56" s="1" t="s">
@@ -5399,7 +5417,7 @@
       <c r="A57" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B57" s="29" t="s">
+      <c r="B57" s="24" t="s">
         <v>482</v>
       </c>
       <c r="C57" s="1" t="s">
@@ -5456,7 +5474,7 @@
       <c r="A58" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B58" s="29" t="s">
+      <c r="B58" s="24" t="s">
         <v>69</v>
       </c>
       <c r="C58" s="1" t="s">
@@ -5509,56 +5527,17 @@
         <v>41</v>
       </c>
     </row>
-    <row r="59" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="32"/>
-      <c r="B59" s="33"/>
-      <c r="E59" s="30"/>
-      <c r="F59" s="22"/>
-      <c r="I59" s="22"/>
-      <c r="J59" s="22"/>
-      <c r="K59" s="22"/>
-      <c r="L59" s="22"/>
-      <c r="M59" s="22"/>
-      <c r="N59" s="22"/>
-      <c r="O59" s="22"/>
-      <c r="P59" s="22"/>
-      <c r="Q59" s="22"/>
-      <c r="R59" s="31"/>
-      <c r="S59" s="22"/>
-    </row>
-    <row r="60" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="34"/>
-      <c r="B60" s="33"/>
-      <c r="E60" s="30"/>
-      <c r="F60" s="22"/>
-      <c r="I60" s="22"/>
-      <c r="J60" s="22"/>
-      <c r="K60" s="22"/>
-      <c r="L60" s="22"/>
-      <c r="M60" s="22"/>
-      <c r="N60" s="22"/>
-      <c r="O60" s="22"/>
-      <c r="P60" s="22"/>
-      <c r="Q60" s="22"/>
-      <c r="R60" s="31"/>
-      <c r="S60" s="22"/>
-    </row>
-    <row r="61" spans="1:21" s="21" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="35"/>
-      <c r="B61" s="33"/>
-      <c r="E61" s="30"/>
-      <c r="F61" s="22"/>
-      <c r="I61" s="22"/>
-      <c r="J61" s="22"/>
-      <c r="K61" s="22"/>
-      <c r="L61" s="22"/>
-      <c r="M61" s="22"/>
-      <c r="N61" s="22"/>
-      <c r="O61" s="22"/>
-      <c r="P61" s="22"/>
-      <c r="Q61" s="22"/>
-      <c r="R61" s="31"/>
-      <c r="S61" s="22"/>
+    <row r="59" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A59" s="26"/>
+      <c r="E59" s="25"/>
+    </row>
+    <row r="60" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A60" s="27"/>
+      <c r="E60" s="25"/>
+    </row>
+    <row r="61" spans="1:21" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="28"/>
+      <c r="E61" s="25"/>
     </row>
   </sheetData>
   <dataValidations xWindow="185" yWindow="923" count="12">
@@ -5655,51 +5634,53 @@
     <hyperlink ref="E34" r:id="rId64" xr:uid="{3D68E0F6-565A-4E31-8041-14A4E4AAA026}"/>
     <hyperlink ref="E5" r:id="rId65" xr:uid="{EF1D420F-18EF-4E76-89A3-98850C9AF20C}"/>
     <hyperlink ref="E35" r:id="rId66" xr:uid="{F78DA305-9BB5-4F2E-B4F8-66EC8FBDDA3D}"/>
-    <hyperlink ref="E11" r:id="rId67" xr:uid="{8F612C67-B290-475F-A329-18B4A1CD494F}"/>
-    <hyperlink ref="E36" r:id="rId68" xr:uid="{34B32381-DA3D-48A1-8F3A-7BA553623903}"/>
-    <hyperlink ref="E37" r:id="rId69" xr:uid="{45465AA5-EEE0-48FC-9065-53047723500D}"/>
-    <hyperlink ref="E38" r:id="rId70" xr:uid="{13BB9942-A405-4DA2-8E06-01F90B4BD748}"/>
-    <hyperlink ref="E6" r:id="rId71" xr:uid="{DA4BEBE2-080E-4CD9-B20D-9A66E0B9BA0E}"/>
-    <hyperlink ref="E2" r:id="rId72" xr:uid="{2A421EFC-5CE1-4915-BCFF-E0F180BC7805}"/>
-    <hyperlink ref="E12" r:id="rId73" xr:uid="{9BAD52EC-0FBB-47D0-B299-98976A4A44C1}"/>
-    <hyperlink ref="E13" r:id="rId74" xr:uid="{BBB29648-EE03-4690-B8CF-7336712FAED6}"/>
-    <hyperlink ref="E3" r:id="rId75" xr:uid="{02DC2D59-84BF-4EEB-AE0B-79A2F174ED4E}"/>
-    <hyperlink ref="E39" r:id="rId76" xr:uid="{A63C04C4-8DD9-435D-ABF9-0203E47DF1B0}"/>
-    <hyperlink ref="E40" r:id="rId77" xr:uid="{8E647A81-A99D-4893-8BBE-EA2D0B10E098}"/>
-    <hyperlink ref="E41" r:id="rId78" xr:uid="{C9CED6DD-2DA0-41FC-871A-F66D82DD880B}"/>
-    <hyperlink ref="E14" r:id="rId79" xr:uid="{2E33A0D8-379C-435E-914F-1511B519A04E}"/>
-    <hyperlink ref="E4" r:id="rId80" xr:uid="{28D87A6B-7FF4-40B3-B258-618F4D30BC9B}"/>
-    <hyperlink ref="E15" r:id="rId81" xr:uid="{25D99204-4613-42A1-BE9B-F2E5D561C894}"/>
-    <hyperlink ref="E16" r:id="rId82" xr:uid="{EB604F45-7F62-4D95-87A0-7C607F70EEE6}"/>
-    <hyperlink ref="E42" r:id="rId83" xr:uid="{FF0F238A-0D26-48C4-A15F-7954889B76EF}"/>
-    <hyperlink ref="E43" r:id="rId84" xr:uid="{60B932FB-29EC-45F2-B889-1CB79A7CA2CB}"/>
-    <hyperlink ref="E44" r:id="rId85" xr:uid="{6A9F5AC2-0769-4F65-A1B3-C7B6B78865CF}"/>
-    <hyperlink ref="E17" r:id="rId86" xr:uid="{8F8CC71E-CB4F-469E-8417-A15A6E522D48}"/>
-    <hyperlink ref="E45" r:id="rId87" xr:uid="{70588B6D-86C2-4E9D-A653-EB43F4458978}"/>
-    <hyperlink ref="E18" r:id="rId88" xr:uid="{2BC13BFC-19BE-477A-82E0-7D14CED900F5}"/>
-    <hyperlink ref="E46" r:id="rId89" xr:uid="{7A331BB3-C033-4479-BE55-986C3D9F9A53}"/>
-    <hyperlink ref="E47" r:id="rId90" xr:uid="{9D770BB2-4EC1-4C1B-9178-82ADFA28631B}"/>
-    <hyperlink ref="E7" r:id="rId91" xr:uid="{9BCD1D34-3807-4EFF-9AFB-1B2D272BAC40}"/>
-    <hyperlink ref="E48" r:id="rId92" xr:uid="{D7E4C853-E250-43E6-9D4D-F09FCBFF6B2F}"/>
-    <hyperlink ref="E49" r:id="rId93" xr:uid="{74D7670D-4811-4714-AC93-1B08F70715DA}"/>
-    <hyperlink ref="E19" r:id="rId94" xr:uid="{CB748B89-0123-4681-825A-E27A0BE8ECB1}"/>
-    <hyperlink ref="E50" r:id="rId95" xr:uid="{A29855BD-159B-419E-AEF2-13C042924D47}"/>
-    <hyperlink ref="E51" r:id="rId96" xr:uid="{4D3EFA2A-19FF-4AD8-84E1-C8E13C595478}"/>
-    <hyperlink ref="E53" r:id="rId97" xr:uid="{A4C956F3-167F-4BD7-A91C-26AD208A0BD1}"/>
-    <hyperlink ref="E54" r:id="rId98" xr:uid="{1749D594-EE49-4E34-B8D1-987FAE0B65C9}"/>
-    <hyperlink ref="E56" r:id="rId99" xr:uid="{1380FF99-EF25-4839-8AF5-637A67A7D467}"/>
-    <hyperlink ref="E57" r:id="rId100" xr:uid="{4E15A300-DD30-44C2-BA8F-B49EEC02963B}"/>
-    <hyperlink ref="E58" r:id="rId101" xr:uid="{0F99CB0B-4B4B-4B69-9AC3-D56535324B5D}"/>
-    <hyperlink ref="E20" r:id="rId102" xr:uid="{D941B546-8A6E-4F9C-AEA8-DF3FB2FD1934}"/>
-    <hyperlink ref="E21" r:id="rId103" xr:uid="{4F41EEAE-E6DF-4432-A83D-08B8DBD75934}"/>
-    <hyperlink ref="E22" r:id="rId104" xr:uid="{1E3794A4-06A0-428E-B3C5-B6CF6637ACB4}"/>
-    <hyperlink ref="F56" r:id="rId105" xr:uid="{435B592D-DD21-4EC5-9AFF-18B7F3BB085D}"/>
-    <hyperlink ref="F22" r:id="rId106" xr:uid="{9242EECC-BD31-44D9-90EB-51E2B0A20F91}"/>
-    <hyperlink ref="F21" r:id="rId107" xr:uid="{E6226532-F402-4D02-8A51-FC5F911E486B}"/>
+    <hyperlink ref="E36" r:id="rId67" xr:uid="{34B32381-DA3D-48A1-8F3A-7BA553623903}"/>
+    <hyperlink ref="E37" r:id="rId68" xr:uid="{45465AA5-EEE0-48FC-9065-53047723500D}"/>
+    <hyperlink ref="E38" r:id="rId69" xr:uid="{13BB9942-A405-4DA2-8E06-01F90B4BD748}"/>
+    <hyperlink ref="E6" r:id="rId70" xr:uid="{DA4BEBE2-080E-4CD9-B20D-9A66E0B9BA0E}"/>
+    <hyperlink ref="E2" r:id="rId71" xr:uid="{2A421EFC-5CE1-4915-BCFF-E0F180BC7805}"/>
+    <hyperlink ref="E12" r:id="rId72" xr:uid="{9BAD52EC-0FBB-47D0-B299-98976A4A44C1}"/>
+    <hyperlink ref="E13" r:id="rId73" xr:uid="{BBB29648-EE03-4690-B8CF-7336712FAED6}"/>
+    <hyperlink ref="E3" r:id="rId74" xr:uid="{02DC2D59-84BF-4EEB-AE0B-79A2F174ED4E}"/>
+    <hyperlink ref="E39" r:id="rId75" xr:uid="{A63C04C4-8DD9-435D-ABF9-0203E47DF1B0}"/>
+    <hyperlink ref="E40" r:id="rId76" xr:uid="{8E647A81-A99D-4893-8BBE-EA2D0B10E098}"/>
+    <hyperlink ref="E14" r:id="rId77" xr:uid="{2E33A0D8-379C-435E-914F-1511B519A04E}"/>
+    <hyperlink ref="E4" r:id="rId78" xr:uid="{28D87A6B-7FF4-40B3-B258-618F4D30BC9B}"/>
+    <hyperlink ref="E16" r:id="rId79" xr:uid="{EB604F45-7F62-4D95-87A0-7C607F70EEE6}"/>
+    <hyperlink ref="E42" r:id="rId80" xr:uid="{FF0F238A-0D26-48C4-A15F-7954889B76EF}"/>
+    <hyperlink ref="E44" r:id="rId81" xr:uid="{6A9F5AC2-0769-4F65-A1B3-C7B6B78865CF}"/>
+    <hyperlink ref="E17" r:id="rId82" xr:uid="{8F8CC71E-CB4F-469E-8417-A15A6E522D48}"/>
+    <hyperlink ref="E45" r:id="rId83" xr:uid="{70588B6D-86C2-4E9D-A653-EB43F4458978}"/>
+    <hyperlink ref="E18" r:id="rId84" xr:uid="{2BC13BFC-19BE-477A-82E0-7D14CED900F5}"/>
+    <hyperlink ref="E46" r:id="rId85" xr:uid="{7A331BB3-C033-4479-BE55-986C3D9F9A53}"/>
+    <hyperlink ref="E47" r:id="rId86" xr:uid="{9D770BB2-4EC1-4C1B-9178-82ADFA28631B}"/>
+    <hyperlink ref="E7" r:id="rId87" xr:uid="{9BCD1D34-3807-4EFF-9AFB-1B2D272BAC40}"/>
+    <hyperlink ref="E48" r:id="rId88" xr:uid="{D7E4C853-E250-43E6-9D4D-F09FCBFF6B2F}"/>
+    <hyperlink ref="E49" r:id="rId89" xr:uid="{74D7670D-4811-4714-AC93-1B08F70715DA}"/>
+    <hyperlink ref="E19" r:id="rId90" xr:uid="{CB748B89-0123-4681-825A-E27A0BE8ECB1}"/>
+    <hyperlink ref="E51" r:id="rId91" xr:uid="{4D3EFA2A-19FF-4AD8-84E1-C8E13C595478}"/>
+    <hyperlink ref="E53" r:id="rId92" xr:uid="{A4C956F3-167F-4BD7-A91C-26AD208A0BD1}"/>
+    <hyperlink ref="E54" r:id="rId93" xr:uid="{1749D594-EE49-4E34-B8D1-987FAE0B65C9}"/>
+    <hyperlink ref="E56" r:id="rId94" xr:uid="{1380FF99-EF25-4839-8AF5-637A67A7D467}"/>
+    <hyperlink ref="E57" r:id="rId95" xr:uid="{4E15A300-DD30-44C2-BA8F-B49EEC02963B}"/>
+    <hyperlink ref="E58" r:id="rId96" xr:uid="{0F99CB0B-4B4B-4B69-9AC3-D56535324B5D}"/>
+    <hyperlink ref="E20" r:id="rId97" xr:uid="{D941B546-8A6E-4F9C-AEA8-DF3FB2FD1934}"/>
+    <hyperlink ref="E21" r:id="rId98" xr:uid="{4F41EEAE-E6DF-4432-A83D-08B8DBD75934}"/>
+    <hyperlink ref="E22" r:id="rId99" xr:uid="{1E3794A4-06A0-428E-B3C5-B6CF6637ACB4}"/>
+    <hyperlink ref="F56" r:id="rId100" xr:uid="{435B592D-DD21-4EC5-9AFF-18B7F3BB085D}"/>
+    <hyperlink ref="F22" r:id="rId101" xr:uid="{9242EECC-BD31-44D9-90EB-51E2B0A20F91}"/>
+    <hyperlink ref="F21" r:id="rId102" xr:uid="{E6226532-F402-4D02-8A51-FC5F911E486B}"/>
+    <hyperlink ref="E15" r:id="rId103" xr:uid="{25D99204-4613-42A1-BE9B-F2E5D561C894}"/>
+    <hyperlink ref="E11" r:id="rId104" xr:uid="{8F612C67-B290-475F-A329-18B4A1CD494F}"/>
+    <hyperlink ref="E41" r:id="rId105" xr:uid="{C9CED6DD-2DA0-41FC-871A-F66D82DD880B}"/>
+    <hyperlink ref="E43" r:id="rId106" xr:uid="{60B932FB-29EC-45F2-B889-1CB79A7CA2CB}"/>
+    <hyperlink ref="E50" r:id="rId107" xr:uid="{A29855BD-159B-419E-AEF2-13C042924D47}"/>
+    <hyperlink ref="E33" r:id="rId108" xr:uid="{8075B8C8-FB88-7B49-BD90-E19F35481EB2}"/>
+    <hyperlink ref="E52" r:id="rId109" xr:uid="{D13B153E-E756-3347-A1AB-AB3EE4BA2858}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId108"/>
+    <tablePart r:id="rId110"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -7109,7 +7090,7 @@
       <c r="A25" s="14" t="s">
         <v>309</v>
       </c>
-      <c r="B25" s="29" t="s">
+      <c r="B25" s="24" t="s">
         <v>453</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -7169,7 +7150,7 @@
       <c r="A26" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="29" t="s">
+      <c r="B26" s="24" t="s">
         <v>454</v>
       </c>
       <c r="C26" s="1" t="s">
@@ -7226,7 +7207,7 @@
       <c r="A27" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="24" t="s">
         <v>455</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -7283,7 +7264,7 @@
       <c r="A28" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="29" t="s">
+      <c r="B28" s="24" t="s">
         <v>456</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -7337,7 +7318,7 @@
       <c r="A29" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B29" s="29" t="s">
+      <c r="B29" s="24" t="s">
         <v>457</v>
       </c>
       <c r="C29" s="1" t="s">
@@ -7391,7 +7372,7 @@
       <c r="A30" s="14" t="s">
         <v>309</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="24" t="s">
         <v>458</v>
       </c>
       <c r="C30" s="1" t="s">
@@ -7448,7 +7429,7 @@
       <c r="A31" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="24" t="s">
         <v>459</v>
       </c>
       <c r="C31" s="1" t="s">
@@ -7506,7 +7487,7 @@
       <c r="A32" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B32" s="29" t="s">
+      <c r="B32" s="24" t="s">
         <v>460</v>
       </c>
       <c r="C32" s="1" t="s">
@@ -7563,7 +7544,7 @@
       <c r="A33" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="24" t="s">
         <v>461</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -7620,7 +7601,7 @@
       <c r="A34" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B34" s="29" t="s">
+      <c r="B34" s="24" t="s">
         <v>462</v>
       </c>
       <c r="C34" s="1" t="s">
@@ -7680,7 +7661,7 @@
       <c r="A35" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B35" s="29" t="s">
+      <c r="B35" s="24" t="s">
         <v>463</v>
       </c>
       <c r="C35" s="1" t="s">
@@ -7734,7 +7715,7 @@
       <c r="A36" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B36" s="29" t="s">
+      <c r="B36" s="24" t="s">
         <v>464</v>
       </c>
       <c r="C36" s="1" t="s">
@@ -7791,7 +7772,7 @@
       <c r="A37" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B37" s="29" t="s">
+      <c r="B37" s="24" t="s">
         <v>465</v>
       </c>
       <c r="C37" s="1" t="s">
@@ -7848,7 +7829,7 @@
       <c r="A38" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B38" s="29" t="s">
+      <c r="B38" s="24" t="s">
         <v>466</v>
       </c>
       <c r="C38" s="1" t="s">
@@ -7898,7 +7879,7 @@
       <c r="A39" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B39" s="29" t="s">
+      <c r="B39" s="24" t="s">
         <v>467</v>
       </c>
       <c r="C39" s="1" t="s">
@@ -7955,7 +7936,7 @@
       <c r="A40" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B40" s="29" t="s">
+      <c r="B40" s="24" t="s">
         <v>468</v>
       </c>
       <c r="C40" s="1" t="s">
@@ -8009,7 +7990,7 @@
       <c r="A41" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="24" t="s">
         <v>469</v>
       </c>
       <c r="C41" s="1" t="s">
@@ -8067,7 +8048,7 @@
       <c r="A42" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B42" s="29" t="s">
+      <c r="B42" s="24" t="s">
         <v>470</v>
       </c>
       <c r="C42" s="1" t="s">
@@ -8124,7 +8105,7 @@
       <c r="A43" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B43" s="24" t="s">
         <v>471</v>
       </c>
       <c r="C43" s="1" t="s">
@@ -8174,7 +8155,7 @@
       <c r="A44" s="17" t="s">
         <v>390</v>
       </c>
-      <c r="B44" s="29" t="s">
+      <c r="B44" s="24" t="s">
         <v>472</v>
       </c>
       <c r="C44" s="1" t="s">
@@ -8222,7 +8203,7 @@
       <c r="A45" s="17" t="s">
         <v>390</v>
       </c>
-      <c r="B45" s="29" t="s">
+      <c r="B45" s="24" t="s">
         <v>473</v>
       </c>
       <c r="C45" s="1" t="s">
@@ -8273,7 +8254,7 @@
       <c r="A46" s="15" t="s">
         <v>403</v>
       </c>
-      <c r="B46" s="29" t="s">
+      <c r="B46" s="24" t="s">
         <v>474</v>
       </c>
       <c r="C46" s="1" t="s">
@@ -8330,7 +8311,7 @@
       <c r="A47" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B47" s="24" t="s">
         <v>475</v>
       </c>
       <c r="C47" s="1" t="s">
@@ -8390,7 +8371,7 @@
       <c r="A48" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="29" t="s">
+      <c r="B48" s="24" t="s">
         <v>476</v>
       </c>
       <c r="C48" s="1" t="s">
@@ -8447,7 +8428,7 @@
       <c r="A49" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B49" s="29" t="s">
+      <c r="B49" s="24" t="s">
         <v>477</v>
       </c>
       <c r="C49" s="1" t="s">
@@ -8496,7 +8477,7 @@
       <c r="A50" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="29" t="s">
+      <c r="B50" s="24" t="s">
         <v>478</v>
       </c>
       <c r="C50" s="1" t="s">
@@ -8551,7 +8532,7 @@
       <c r="A51" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B51" s="29" t="s">
+      <c r="B51" s="24" t="s">
         <v>479</v>
       </c>
       <c r="C51" s="1" t="s">
@@ -8604,7 +8585,7 @@
       <c r="A52" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B52" s="29" t="s">
+      <c r="B52" s="24" t="s">
         <v>480</v>
       </c>
       <c r="C52" s="1" t="s">
@@ -8661,7 +8642,7 @@
       <c r="A53" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B53" s="29" t="s">
+      <c r="B53" s="24" t="s">
         <v>481</v>
       </c>
       <c r="C53" s="1" t="s">
@@ -8720,7 +8701,7 @@
       <c r="A54" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B54" s="29" t="s">
+      <c r="B54" s="24" t="s">
         <v>482</v>
       </c>
       <c r="C54" s="1" t="s">
@@ -8777,7 +8758,7 @@
       <c r="A55" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B55" s="29" t="s">
+      <c r="B55" s="24" t="s">
         <v>69</v>
       </c>
       <c r="C55" s="1" t="s">
@@ -8834,7 +8815,7 @@
       <c r="A56" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B56" s="29" t="s">
+      <c r="B56" s="24" t="s">
         <v>483</v>
       </c>
       <c r="C56" s="1" t="s">
@@ -8888,7 +8869,7 @@
       <c r="A57" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B57" s="29" t="s">
+      <c r="B57" s="24" t="s">
         <v>484</v>
       </c>
       <c r="C57" s="1" t="s">
@@ -8947,7 +8928,7 @@
       <c r="A58" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B58" s="29" t="s">
+      <c r="B58" s="24" t="s">
         <v>485</v>
       </c>
       <c r="C58" s="1" t="s">
@@ -9003,15 +8984,15 @@
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A59" s="26"/>
-      <c r="B59" s="29" t="s">
+      <c r="A59" s="21"/>
+      <c r="B59" s="24" t="s">
         <v>486</v>
       </c>
       <c r="C59" s="1"/>
       <c r="D59" s="9"/>
-      <c r="E59" s="27"/>
+      <c r="E59" s="22"/>
       <c r="F59" s="7"/>
-      <c r="G59" s="28"/>
+      <c r="G59" s="23"/>
       <c r="H59" s="1"/>
       <c r="I59"/>
       <c r="O59" s="4"/>
@@ -9024,19 +9005,19 @@
       <c r="A61" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="B61" s="23"/>
+      <c r="B61" s="14"/>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A62" s="19" t="s">
         <v>426</v>
       </c>
-      <c r="B62" s="24"/>
+      <c r="B62" s="15"/>
     </row>
     <row r="63" spans="1:21" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="20" t="s">
         <v>427</v>
       </c>
-      <c r="B63" s="25"/>
+      <c r="B63" s="13"/>
     </row>
   </sheetData>
   <dataValidations count="12">
@@ -9236,32 +9217,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <ArtifactsRequested_x003f_ xmlns="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e">Yes</ArtifactsRequested_x003f_>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="6f04fd38-88d0-493d-bcfe-f0680152bc54" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="c3a201dd-47de-4cb5-b1b8-fb4eacb25aeb" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010067084DD94AAF9F49A29187A8281A736B" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="31370f96594e886cf5a1a287283c7112">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e" xmlns:ns3="9843afbf-a983-44da-9ef0-770fe2475dd9" xmlns:ns4="6f04fd38-88d0-493d-bcfe-f0680152bc54" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd273aee41ba6857014841f4b535fddc" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e"/>
@@ -9535,34 +9490,33 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91E5FD91-6CDF-4778-8B48-65EB30B9BE76}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e"/>
-    <ds:schemaRef ds:uri="6f04fd38-88d0-493d-bcfe-f0680152bc54"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="c3a201dd-47de-4cb5-b1b8-fb4eacb25aeb" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4C0E0DC-1A45-4E37-9177-6BF15AAC155D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2749A39F-5866-4570-A7EA-0749A01EC9F3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <ArtifactsRequested_x003f_ xmlns="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e">Yes</ArtifactsRequested_x003f_>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="6f04fd38-88d0-493d-bcfe-f0680152bc54" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08ABF4CA-0893-4703-B384-163F0489B58B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9580,4 +9534,31 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2749A39F-5866-4570-A7EA-0749A01EC9F3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4C0E0DC-1A45-4E37-9177-6BF15AAC155D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91E5FD91-6CDF-4778-8B48-65EB30B9BE76}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e"/>
+    <ds:schemaRef ds:uri="6f04fd38-88d0-493d-bcfe-f0680152bc54"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updates to accomodate NY info
</commit_message>
<xml_diff>
--- a/updatedMemberData.xlsx
+++ b/updatedMemberData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madmarshall/Documents/medicaidOversightMap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D65A340F-9EFD-5849-88C1-447E468EF906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3B4BE4-EB0E-C846-8EB1-24581645C0F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4420" yWindow="960" windowWidth="21400" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4305,7 +4305,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A37" s="13" t="s">
-        <v>20</v>
+        <v>288</v>
       </c>
       <c r="B37" s="24" t="s">
         <v>463</v>

</xml_diff>

<commit_message>
Update moved file names; implement edits from for select state agency names
</commit_message>
<xml_diff>
--- a/updatedMemberData.xlsx
+++ b/updatedMemberData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madmarshall/Documents/medicaidOversightMap/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madmarshall/Documents/01_ASTHO/03_HRSA-NOSLO/medicaidOversightMap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3B4BE4-EB0E-C846-8EB1-24581645C0F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718BADA5-9714-6742-9432-D4257B2E4DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="960" windowWidth="21400" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6040" yWindow="800" windowWidth="22160" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1960" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1975" uniqueCount="507">
   <si>
     <t>Oversight?</t>
   </si>
@@ -1523,6 +1523,42 @@
   </si>
   <si>
     <t>https://www.chfs.ky.gov/services/Pages/search.aspx</t>
+  </si>
+  <si>
+    <t>Idaho Division of Public Health</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maryland Department of Health </t>
+  </si>
+  <si>
+    <t>https://health.maryland.gov/Pages/Home.aspx</t>
+  </si>
+  <si>
+    <t>MD-DOH</t>
+  </si>
+  <si>
+    <t>Seshamani, Meena</t>
+  </si>
+  <si>
+    <t>Sullivan, Meg</t>
+  </si>
+  <si>
+    <t>https://health.maryland.gov/iac/Documents/MDH%20Organization%20Chart%20-%20060525.pdf</t>
+  </si>
+  <si>
+    <t>Maryland</t>
+  </si>
+  <si>
+    <t>202</t>
+  </si>
+  <si>
+    <t>New Hampshire Department of Health &amp; Human Services, Division of Public Health</t>
+  </si>
+  <si>
+    <t>Wisconsin Department of Health Services, Division of Public Health</t>
+  </si>
+  <si>
+    <t>Delaware Department of Health and Social Services, Division of Public Health</t>
   </si>
 </sst>
 </file>
@@ -1532,7 +1568,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
@@ -1548,6 +1584,11 @@
       <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1606,7 +1647,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1693,12 +1734,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF44B3E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF44B3E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1729,6 +1781,9 @@
     <xf numFmtId="22" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1863,10 +1918,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:U58" totalsRowShown="0">
-  <autoFilter ref="A1:U58" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U58">
-    <sortCondition ref="B1:B58"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:U59" totalsRowShown="0">
+  <autoFilter ref="A1:U59" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U59">
+    <sortCondition ref="B1:B59"/>
   </sortState>
   <tableColumns count="21">
     <tableColumn id="24" xr3:uid="{EC3A8AE4-1AEA-44FE-9DAE-C845A25235D5}" name="Oversight?" dataDxfId="13"/>
@@ -2246,7 +2301,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="dataSheet"/>
-  <dimension ref="A1:U61"/>
+  <dimension ref="A1:U62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="42.83203125" style="2" customWidth="1"/>
@@ -2842,7 +2897,7 @@
         <v>438</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>281</v>
+        <v>506</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>260</v>
@@ -3227,7 +3282,7 @@
         <v>445</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>295</v>
+        <v>495</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>260</v>
@@ -4137,7 +4192,7 @@
         <v>460</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>362</v>
+        <v>504</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>260</v>
@@ -4314,7 +4369,7 @@
         <v>146</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>22</v>
+        <v>260</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>147</v>
@@ -5130,7 +5185,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A52" s="13" t="s">
-        <v>20</v>
+        <v>258</v>
       </c>
       <c r="B52" s="24" t="s">
         <v>480</v>
@@ -5139,7 +5194,7 @@
         <v>204</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>22</v>
+        <v>260</v>
       </c>
       <c r="E52" s="4" t="s">
         <v>205</v>
@@ -5413,50 +5468,43 @@
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A57" s="15" t="s">
-        <v>258</v>
+      <c r="A57" s="21" t="s">
+        <v>309</v>
       </c>
       <c r="B57" s="24" t="s">
-        <v>484</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="D57" s="9" t="s">
+        <v>502</v>
+      </c>
+      <c r="C57" s="30" t="s">
+        <v>496</v>
+      </c>
+      <c r="D57" s="30" t="s">
         <v>260</v>
       </c>
-      <c r="E57" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="F57" s="7" t="s">
-        <v>262</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>24</v>
+      <c r="E57" s="31" t="s">
+        <v>497</v>
+      </c>
+      <c r="F57" s="7"/>
+      <c r="G57" s="23" t="s">
+        <v>503</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="I57" t="s">
-        <v>37</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="M57" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="N57" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="O57" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="P57" s="1" t="s">
-        <v>267</v>
+        <v>498</v>
+      </c>
+      <c r="I57"/>
+      <c r="J57" s="30" t="s">
+        <v>499</v>
+      </c>
+      <c r="K57" s="30" t="s">
+        <v>500</v>
+      </c>
+      <c r="O57" s="32" t="s">
+        <v>501</v>
+      </c>
+      <c r="P57" s="30" t="s">
+        <v>499</v>
       </c>
       <c r="Q57" s="3">
-        <v>5822434</v>
+        <v>6265347</v>
       </c>
       <c r="R57" s="1" t="s">
         <v>30</v>
@@ -5465,108 +5513,167 @@
         <v>219</v>
       </c>
       <c r="T57" t="s">
-        <v>32</v>
+        <v>219</v>
       </c>
       <c r="U57" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A58" s="15" t="s">
         <v>258</v>
       </c>
       <c r="B58" s="24" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>417</v>
+        <v>505</v>
       </c>
       <c r="D58" s="9" t="s">
         <v>260</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>418</v>
+        <v>261</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>419</v>
+        <v>262</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>24</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>420</v>
+        <v>263</v>
       </c>
       <c r="I58" t="s">
-        <v>168</v>
+        <v>37</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="K58" s="1" t="s">
-        <v>422</v>
+        <v>264</v>
+      </c>
+      <c r="M58" s="1" t="s">
+        <v>265</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>423</v>
+        <v>266</v>
       </c>
       <c r="O58" s="4" t="s">
-        <v>418</v>
+        <v>261</v>
       </c>
       <c r="P58" s="1" t="s">
-        <v>424</v>
+        <v>267</v>
       </c>
       <c r="Q58" s="3">
-        <v>578759</v>
+        <v>5822434</v>
       </c>
       <c r="R58" s="1" t="s">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="S58" t="s">
-        <v>71</v>
+        <v>219</v>
       </c>
       <c r="T58" t="s">
         <v>32</v>
       </c>
       <c r="U58" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="B59" s="24" t="s">
+        <v>485</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="F59" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="I59" t="s">
+        <v>168</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="K59" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="N59" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="O59" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="P59" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="Q59" s="3">
+        <v>578759</v>
+      </c>
+      <c r="R59" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="S59" t="s">
+        <v>71</v>
+      </c>
+      <c r="T59" t="s">
+        <v>32</v>
+      </c>
+      <c r="U59" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A59" s="26"/>
-      <c r="E59" s="25"/>
-    </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A60" s="27"/>
+      <c r="A60" s="26"/>
       <c r="E60" s="25"/>
     </row>
-    <row r="61" spans="1:21" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="28"/>
+    <row r="61" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A61" s="27"/>
       <c r="E61" s="25"/>
+    </row>
+    <row r="62" spans="1:21" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="28"/>
+      <c r="E62" s="25"/>
     </row>
   </sheetData>
   <dataValidations xWindow="185" yWindow="923" count="12">
-    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 20 characters long." promptTitle="Text" prompt="Maximum Length: 20 characters." sqref="H2:H58 I59:I1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 20 characters long." promptTitle="Text" prompt="Maximum Length: 20 characters." sqref="H2:H59 I60:I1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>20</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="lessThanOrEqual" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 160 characters long." promptTitle="Text (required)" prompt="Maximum Length: 160 characters." sqref="C2:C58" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="textLength" operator="lessThanOrEqual" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 160 characters long." promptTitle="Text (required)" prompt="Maximum Length: 160 characters." sqref="C2:C56 C58:C59" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>160</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="MultiSelect Option set" prompt="Enter Option Set values as semicolon separated." sqref="I2:I58 S2:U58 T59:V1048576 H59:J1048576" xr:uid="{00000000-0002-0000-0000-000006000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This S/THO record must already exist in Microsoft Dynamics 365 or in this source file." sqref="J2:J58 K59:K1048576" xr:uid="{00000000-0002-0000-0000-000007000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This S/THO Designee record must already exist in Microsoft Dynamics 365 or in this source file." sqref="K2:K58 L59:L1048576" xr:uid="{00000000-0002-0000-0000-000008000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This S/THO Acting record must already exist in Microsoft Dynamics 365 or in this source file." sqref="L2:L58 M59:M1048576" xr:uid="{00000000-0002-0000-0000-000009000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This S/THO Assistant record must already exist in Microsoft Dynamics 365 or in this source file." sqref="M2:M58 N59:N1048576" xr:uid="{00000000-0002-0000-0000-00000A000000}"/>
-    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 80 characters long." promptTitle="Text" prompt="Maximum Length: 80 characters." sqref="N2:N58 O59:O1048576" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="MultiSelect Option set" prompt="Enter Option Set values as semicolon separated." sqref="I2:I59 S2:U59 T60:V1048576 H60:J1048576" xr:uid="{00000000-0002-0000-0000-000006000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This S/THO record must already exist in Microsoft Dynamics 365 or in this source file." sqref="K60:K1048576 J2:J56 J58:J59" xr:uid="{00000000-0002-0000-0000-000007000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This S/THO Designee record must already exist in Microsoft Dynamics 365 or in this source file." sqref="L60:L1048576 K2:K56 K58:K59" xr:uid="{00000000-0002-0000-0000-000008000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This S/THO Acting record must already exist in Microsoft Dynamics 365 or in this source file." sqref="L2:L59 M60:M1048576" xr:uid="{00000000-0002-0000-0000-000009000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This S/THO Assistant record must already exist in Microsoft Dynamics 365 or in this source file." sqref="M2:M59 N60:N1048576" xr:uid="{00000000-0002-0000-0000-00000A000000}"/>
+    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 80 characters long." promptTitle="Text" prompt="Maximum Length: 80 characters." sqref="N2:N59 O60:O1048576" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>80</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 200 characters long." promptTitle="Text" prompt="Maximum Length: 200 characters." sqref="E2:F58 O2:O58 P59:P1048576" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 200 characters long." promptTitle="Text" prompt="Maximum Length: 200 characters." sqref="P60:P1048576 E58:E59 F2:F59 E2:E56 O2:O56 O58:O59" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>200</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This Secretary of Health record must already exist in Microsoft Dynamics 365 or in this source file." sqref="P2:P58 Q59:Q1048576" xr:uid="{00000000-0002-0000-0000-00000D000000}"/>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value beyond range" error="Population must be a whole number from 0 through 2147483647." promptTitle="Whole number" prompt="Minimum Value: 0._x000d__x000a_Maximum Value: 2147483647._x000d__x000a_  " sqref="Q2:Q58 R59:R1048576" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup" prompt="This Secretary of Health record must already exist in Microsoft Dynamics 365 or in this source file." sqref="Q60:Q1048576 P2:P56 P58:P59" xr:uid="{00000000-0002-0000-0000-00000D000000}"/>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value beyond range" error="Population must be a whole number from 0 through 2147483647." promptTitle="Whole number" prompt="Minimum Value: 0._x000d__x000a_Maximum Value: 2147483647._x000d__x000a_  " sqref="Q2:Q59 R60:R1048576" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>0</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 4 characters long." promptTitle="Text" prompt="Maximum Length: 4 characters." sqref="G2:G58 F59:F1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 4 characters long." promptTitle="Text" prompt="Maximum Length: 4 characters." sqref="G2:G59 F60:F1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>4</formula1>
     </dataValidation>
   </dataValidations>
@@ -5620,8 +5727,8 @@
     <hyperlink ref="O54" r:id="rId47" xr:uid="{D7B0DACD-5FD1-4346-B4E7-958EFDE6DA7C}"/>
     <hyperlink ref="O55" r:id="rId48" xr:uid="{55EB6149-0908-4B53-A043-978695B6AFF2}"/>
     <hyperlink ref="O56" r:id="rId49" xr:uid="{566E4284-EA29-42AE-ADF0-6D11CA2D7918}"/>
-    <hyperlink ref="O57" r:id="rId50" xr:uid="{1F555AFE-78CF-4F3C-9D4D-8A9484A22E05}"/>
-    <hyperlink ref="O58" r:id="rId51" xr:uid="{A07AD047-9BF8-4A20-B9F9-4A6749EA616A}"/>
+    <hyperlink ref="O58" r:id="rId50" xr:uid="{1F555AFE-78CF-4F3C-9D4D-8A9484A22E05}"/>
+    <hyperlink ref="O59" r:id="rId51" xr:uid="{A07AD047-9BF8-4A20-B9F9-4A6749EA616A}"/>
     <hyperlink ref="E2" r:id="rId52" xr:uid="{FEE37E5B-198F-4348-8CCA-D7ED5F656AAC}"/>
     <hyperlink ref="E3" r:id="rId53" xr:uid="{03D7C8ED-BBB4-45E8-BC5C-86ACD2650E41}"/>
     <hyperlink ref="E4" r:id="rId54" xr:uid="{0CC618F9-D07B-4A57-BB30-DA9D9C4F2552}"/>
@@ -5666,11 +5773,11 @@
     <hyperlink ref="E54" r:id="rId93" xr:uid="{4E15A300-DD30-44C2-BA8F-B49EEC02963B}"/>
     <hyperlink ref="E55" r:id="rId94" xr:uid="{0F99CB0B-4B4B-4B69-9AC3-D56535324B5D}"/>
     <hyperlink ref="E56" r:id="rId95" xr:uid="{D941B546-8A6E-4F9C-AEA8-DF3FB2FD1934}"/>
-    <hyperlink ref="E57" r:id="rId96" xr:uid="{4F41EEAE-E6DF-4432-A83D-08B8DBD75934}"/>
-    <hyperlink ref="E58" r:id="rId97" xr:uid="{1E3794A4-06A0-428E-B3C5-B6CF6637ACB4}"/>
+    <hyperlink ref="E58" r:id="rId96" xr:uid="{4F41EEAE-E6DF-4432-A83D-08B8DBD75934}"/>
+    <hyperlink ref="E59" r:id="rId97" xr:uid="{1E3794A4-06A0-428E-B3C5-B6CF6637ACB4}"/>
     <hyperlink ref="F53" r:id="rId98" xr:uid="{435B592D-DD21-4EC5-9AFF-18B7F3BB085D}"/>
-    <hyperlink ref="F58" r:id="rId99" xr:uid="{9242EECC-BD31-44D9-90EB-51E2B0A20F91}"/>
-    <hyperlink ref="F57" r:id="rId100" xr:uid="{E6226532-F402-4D02-8A51-FC5F911E486B}"/>
+    <hyperlink ref="F59" r:id="rId99" xr:uid="{9242EECC-BD31-44D9-90EB-51E2B0A20F91}"/>
+    <hyperlink ref="F58" r:id="rId100" xr:uid="{E6226532-F402-4D02-8A51-FC5F911E486B}"/>
     <hyperlink ref="E33" r:id="rId101" xr:uid="{25D99204-4613-42A1-BE9B-F2E5D561C894}"/>
     <hyperlink ref="E18" r:id="rId102" xr:uid="{8F612C67-B290-475F-A329-18B4A1CD494F}"/>
     <hyperlink ref="E30" r:id="rId103" xr:uid="{C9CED6DD-2DA0-41FC-871A-F66D82DD880B}"/>
@@ -5678,10 +5785,12 @@
     <hyperlink ref="E47" r:id="rId105" xr:uid="{A29855BD-159B-419E-AEF2-13C042924D47}"/>
     <hyperlink ref="E15" r:id="rId106" xr:uid="{8075B8C8-FB88-7B49-BD90-E19F35481EB2}"/>
     <hyperlink ref="E49" r:id="rId107" xr:uid="{D13B153E-E756-3347-A1AB-AB3EE4BA2858}"/>
+    <hyperlink ref="E57" r:id="rId108" xr:uid="{3364B68C-0A03-B94D-9B32-7FFC45828012}"/>
+    <hyperlink ref="O57" r:id="rId109" display="https://health.maryland.gov/iac/Documents/MDH Organization Chart - 060525.pdf" xr:uid="{B213A2ED-7407-3440-A577-14A61D6B769E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId108"/>
+    <tablePart r:id="rId110"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -5690,13 +5799,13 @@
           <x14:formula1>
             <xm:f>hiddenSheet!$A$2:$C$2</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:H58 J59:J1048576</xm:sqref>
+          <xm:sqref>J60:J1048576 F2:H59 D58:E59 D2:E56</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="List Value" error="PHAB Accreditation must be selected from the drop-down list." promptTitle="Option set" prompt="Select a value from the drop-down list." xr:uid="{00000000-0002-0000-0000-00000F000000}">
           <x14:formula1>
             <xm:f>hiddenSheet!$A$3:$B$3</xm:f>
           </x14:formula1>
-          <xm:sqref>R2:R58 S59:S1048576</xm:sqref>
+          <xm:sqref>R2:R59 S60:S1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -9218,6 +9327,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <ArtifactsRequested_x003f_ xmlns="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e">Yes</ArtifactsRequested_x003f_>
@@ -9229,21 +9347,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="c3a201dd-47de-4cb5-b1b8-fb4eacb25aeb" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010067084DD94AAF9F49A29187A8281A736B" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="31370f96594e886cf5a1a287283c7112">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e" xmlns:ns3="9843afbf-a983-44da-9ef0-770fe2475dd9" xmlns:ns4="6f04fd38-88d0-493d-bcfe-f0680152bc54" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd273aee41ba6857014841f4b535fddc" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="c6cb7c5a-edb7-416a-adb1-0d17ade57b9e"/>
@@ -9517,7 +9621,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="c3a201dd-47de-4cb5-b1b8-fb4eacb25aeb" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4C0E0DC-1A45-4E37-9177-6BF15AAC155D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91E5FD91-6CDF-4778-8B48-65EB30B9BE76}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9528,23 +9645,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4C0E0DC-1A45-4E37-9177-6BF15AAC155D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2749A39F-5866-4570-A7EA-0749A01EC9F3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08ABF4CA-0893-4703-B384-163F0489B58B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9562,4 +9663,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2749A39F-5866-4570-A7EA-0749A01EC9F3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>